<commit_message>
ASEC median anchor: endpoint design, ASEC income medians and diagnostics
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/tables/universal_sm_hybrid/hybrid_by_route.xlsx
+++ b/output/tables/universal_sm_hybrid/hybrid_by_route.xlsx
@@ -395,22 +395,22 @@
         <v>7</v>
       </c>
       <c r="B2" t="n">
-        <v>1828</v>
+        <v>1644</v>
       </c>
       <c r="C2" t="n">
-        <v>18.4891458945881</v>
+        <v>19.8589494402934</v>
       </c>
       <c r="D2" t="n">
-        <v>41301.1279882902</v>
+        <v>45113.4781875258</v>
       </c>
       <c r="E2" t="n">
-        <v>65.7772203210134</v>
+        <v>60.7932375728129</v>
       </c>
       <c r="F2" t="n">
-        <v>9916.42468871174</v>
+        <v>10208.4952791276</v>
       </c>
       <c r="G2" t="n">
-        <v>1848.91458945881</v>
+        <v>1985.89494402934</v>
       </c>
     </row>
     <row r="3">
@@ -418,22 +418,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="n">
-        <v>2743</v>
+        <v>2649</v>
       </c>
       <c r="C3" t="n">
-        <v>25.9833265074087</v>
+        <v>29.9235052309671</v>
       </c>
       <c r="D3" t="n">
-        <v>34767.7775508686</v>
+        <v>35149.8171431346</v>
       </c>
       <c r="E3" t="n">
-        <v>84.7042163740556</v>
+        <v>85.4084725658813</v>
       </c>
       <c r="F3" t="n">
-        <v>13949.1949654053</v>
+        <v>16157.9561575226</v>
       </c>
       <c r="G3" t="n">
-        <v>2598.33265074087</v>
+        <v>2992.35052309671</v>
       </c>
     </row>
   </sheetData>

</xml_diff>